<commit_message>
feat: add application import preview modal
</commit_message>
<xml_diff>
--- a/prompt/liste_des_demandes_import.xlsx
+++ b/prompt/liste_des_demandes_import.xlsx
@@ -11,7 +11,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="36" uniqueCount="30">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="50" uniqueCount="42">
   <si>
     <t>N°</t>
   </si>
@@ -101,6 +101,42 @@
   </si>
   <si>
     <t>REF-IMP-004</t>
+  </si>
+  <si>
+    <t>Fatou</t>
+  </si>
+  <si>
+    <t>05/04/2001</t>
+  </si>
+  <si>
+    <t>998877665</t>
+  </si>
+  <si>
+    <t>Yoff Golf Sud, Dakar</t>
+  </si>
+  <si>
+    <t>+221 70 400 40 40</t>
+  </si>
+  <si>
+    <t>REF-767G56</t>
+  </si>
+  <si>
+    <t>Gueye</t>
+  </si>
+  <si>
+    <t>Modou</t>
+  </si>
+  <si>
+    <t/>
+  </si>
+  <si>
+    <t>Dakar, Senegal</t>
+  </si>
+  <si>
+    <t>+221 76 111 22 33</t>
+  </si>
+  <si>
+    <t>REF-IMP-006</t>
   </si>
 </sst>
 </file>
@@ -477,7 +513,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:H5"/>
+  <dimension ref="A1:H7"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <sheetData>
     <row r="1" spans="1:8" x14ac:dyDescent="0.25">
@@ -608,6 +644,58 @@
       </c>
       <c r="H5" t="s">
         <v>29</v>
+      </c>
+    </row>
+    <row r="6" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A6">
+        <v>5</v>
+      </c>
+      <c r="B6" t="s">
+        <v>8</v>
+      </c>
+      <c r="C6" t="s">
+        <v>30</v>
+      </c>
+      <c r="D6" t="s">
+        <v>31</v>
+      </c>
+      <c r="E6" t="s">
+        <v>32</v>
+      </c>
+      <c r="F6" t="s">
+        <v>33</v>
+      </c>
+      <c r="G6" t="s">
+        <v>34</v>
+      </c>
+      <c r="H6" t="s">
+        <v>35</v>
+      </c>
+    </row>
+    <row r="7" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A7">
+        <v>6</v>
+      </c>
+      <c r="B7" t="s">
+        <v>36</v>
+      </c>
+      <c r="C7" t="s">
+        <v>37</v>
+      </c>
+      <c r="D7" t="s">
+        <v>38</v>
+      </c>
+      <c r="E7" t="s">
+        <v>38</v>
+      </c>
+      <c r="F7" t="s">
+        <v>39</v>
+      </c>
+      <c r="G7" t="s">
+        <v>40</v>
+      </c>
+      <c r="H7" t="s">
+        <v>41</v>
       </c>
     </row>
   </sheetData>

</xml_diff>